<commit_message>
Homogénéise les .xlsx équipements des villes avec le référentiel Abidjan mis à jour
Ajoute/synchronise la colonne Ponderation dans chaque {Ville}_amenities.xlsx
par jointure sur le référentiel Abidjan_amenities.xlsx (seul fichier
réellement lu par le pipeline) — ces fichiers par ville ne servent qu'à la
revue/documentation des pondérations, pas au calcul.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/equipements_osm/Douala_amenities.xlsx
+++ b/data/equipements_osm/Douala_amenities.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -428,715 +428,933 @@
           <t>nombre</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Ponderation</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>school</t>
+          <t>university</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>544</v>
+        <v>10</v>
+      </c>
+      <c r="C2" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>fuel</t>
+          <t>hospital</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>168</v>
+        <v>24</v>
+      </c>
+      <c r="C3" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>bank</t>
+          <t>public_building</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>154</v>
+        <v>10</v>
+      </c>
+      <c r="C4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>clinic</t>
+          <t>community_centre</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>108</v>
+        <v>7</v>
+      </c>
+      <c r="C5" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>place_of_worship</t>
+          <t>townhall</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>106</v>
+        <v>8</v>
+      </c>
+      <c r="C6" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>bar</t>
+          <t>marketplace</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>88</v>
+        <v>26</v>
+      </c>
+      <c r="C7" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>pharmacy</t>
+          <t>courthouse</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>87</v>
+        <v>4</v>
+      </c>
+      <c r="C8" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>cinema</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>79</v>
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>veterinary</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>36</v>
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>doctors</t>
+          <t>clinic</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>28</v>
+        <v>108</v>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>marketplace</t>
+          <t>college</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>26</v>
+        <v>8</v>
+      </c>
+      <c r="C12" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>hospital</t>
+          <t>library</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>24</v>
+        <v>1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>police</t>
+          <t>pharmacy</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>24</v>
+        <v>87</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>nightclub</t>
+          <t>school</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>17</v>
+        <v>544</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>drinking_water</t>
+          <t>doctors</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>15</v>
+        <v>28</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>bus_station</t>
+          <t>bank</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>12</v>
+        <v>154</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>kindergarten</t>
+          <t>post_office</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>11</v>
+        <v>4</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cafe</t>
+          <t>social_facility</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>10</v>
+        <v>5</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>university</t>
+          <t>sanitary_dump_station</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>waste_basket</t>
+          <t>lecture_hall</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>public_building</t>
+          <t>watering_place</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>fast_food</t>
+          <t>food_court</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>9</v>
+        <v>2</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>driving_school</t>
+          <t>grave_yard</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>8</v>
+        <v>2</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>college</t>
+          <t>fire_station</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>8</v>
+        <v>2</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>townhall</t>
+          <t>bureau_de_change</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>8</v>
+        <v>2</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>waste_disposal</t>
+          <t>coworking_space</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>8</v>
+        <v>2</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>community_centre</t>
+          <t>water_point</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>7</v>
+        <v>1</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>pub</t>
+          <t>recycling</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>atm</t>
+          <t>taxi</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>nursing_home</t>
+          <t>parcel_locker</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>social_facility</t>
+          <t>bicycle_parking</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>post_office</t>
+          <t>car_wash</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>courthouse</t>
+          <t>car_rental</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>casino</t>
+          <t>bench</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>cinema</t>
+          <t>hookah_lounge</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ice_cream</t>
+          <t>toilets</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>shelter</t>
+          <t>insurance</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>internet_cafe</t>
+          <t>money_transfer</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>lavoir</t>
+          <t>register_office</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>arts_centre</t>
+          <t>ranger_station</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>factory</t>
+          <t>civic</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>vending_machine</t>
+          <t>fountain</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>telephone</t>
+          <t>car_sharing</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>2</v>
       </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>studio</t>
+          <t>shelter</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>car_wash</t>
+          <t>studio</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>2</v>
       </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>car_sharing</t>
+          <t>telephone</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>2</v>
       </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>coworking_space</t>
+          <t>place_of_worship</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2</v>
+        <v>106</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>bureau_de_change</t>
+          <t>bar</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2</v>
+        <v>88</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>fire_station</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2</v>
+        <v>79</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>grave_yard</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2</v>
+        <v>36</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>food_court</t>
+          <t>police</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2</v>
+        <v>24</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>water_point</t>
+          <t>nightclub</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1</v>
+        <v>17</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>sanitary_dump_station</t>
+          <t>drinking_water</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>15</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>watering_place</t>
+          <t>bus_station</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>veterinary</t>
+          <t>kindergarten</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>lecture_hall</t>
+          <t>cafe</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>10</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>taxi</t>
+          <t>waste_basket</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1</v>
+        <v>10</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>parcel_locker</t>
+          <t>fast_food</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1</v>
+        <v>9</v>
+      </c>
+      <c r="C59" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>bicycle_parking</t>
+          <t>driving_school</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>recycling</t>
+          <t>waste_disposal</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="C61" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>car_rental</t>
+          <t>pub</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="C62" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>library</t>
+          <t>atm</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>bench</t>
+          <t>nursing_home</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="C64" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>hookah_lounge</t>
+          <t>casino</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="C65" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>toilets</t>
+          <t>ice_cream</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="C66" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>insurance</t>
+          <t>fuel</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1</v>
+        <v>168</v>
+      </c>
+      <c r="C67" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>money_transfer</t>
+          <t>internet_cafe</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="C68" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>register_office</t>
+          <t>lavoir</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="C69" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ranger_station</t>
+          <t>arts_centre</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="C70" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>civic</t>
+          <t>factory</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>fountain</t>
+          <t>vending_machine</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="C72" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -1147,6 +1365,9 @@
       </c>
       <c r="B73" t="n">
         <v>1</v>
+      </c>
+      <c r="C73" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>